<commit_message>
Add STARS report link to graduation plan and rebalance Spring 2027
Upload stars-report.pdf, sync plan with STARS Fall 2026 registration,
remove duplicate BUAD 281 from Spring 27, spread quant courses, and add
Notes column for load-balancing guidance.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/graduation-plan.xlsx
+++ b/output/graduation-plan.xlsx
@@ -57,7 +57,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -67,7 +67,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -496,6 +496,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -541,6 +542,11 @@
           <t>Cumulative Total</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -562,6 +568,7 @@
           <t>51.0</t>
         </is>
       </c>
+      <c r="H3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -571,32 +578,37 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>BUAD 304</t>
+          <t>BUAD 281</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Organizational Behavior and Leadership</t>
+          <t>Introduction to Managerial Accounting</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Marshall Core</t>
+          <t>Accounting / Marshall Core</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>In progress per STARS (08/15/26)</t>
         </is>
       </c>
     </row>
@@ -604,17 +616,17 @@
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ECON 351</t>
+          <t>BUAD 304</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Microeconomics for Business</t>
+          <t>Organizational Behavior and Leadership</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Marshall Core / Econ</t>
+          <t>Marshall Core</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -624,22 +636,23 @@
       </c>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr"/>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Rel 137</t>
+          <t>ECON 351</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Intro to Islam</t>
+          <t>Microeconomics for Business</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>GE Category B</t>
+          <t>Economics / Marshall Core</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -649,84 +662,91 @@
       </c>
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>HIST 103</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>The Emergence of Modern Europe</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>GE Category B (Humanistic Inquiry)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Spring 2027</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>BUAD 281</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Introduction to Managerial Accounting</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>BUAD 302</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Communication Strategy for Business</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Marshall Core</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>15.0</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>78.0</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr"/>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>BUAD 306</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Business Finance</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Marshall Core</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Rebalanced — lighter than finance/stats stack</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ECON 352</t>
+          <t>GE-C Course</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Macroeconomics for Business</t>
+          <t>Approved Social Analysis (e.g. ANTH 202)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Major Requirement</t>
+          <t>GE Category C</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -736,22 +756,27 @@
       </c>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Fulfills remaining GE-C; non-quant</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>GE-C Course</t>
+          <t>Elective</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Approved Social Analysis Course</t>
+          <t>General Free Elective</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>GE Category C</t>
+          <t>Degree Units</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -761,6 +786,11 @@
       </c>
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Buffer — keeps load at 12 not 15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -770,12 +800,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>BUAD 302</t>
+          <t>BUAD 306</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Communication Strategy for Business</t>
+          <t>Business Finance</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -796,6 +826,11 @@
       <c r="G11" s="4" t="inlineStr">
         <is>
           <t>90.0</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Quant course — paired with macro only</t>
         </is>
       </c>
     </row>
@@ -803,17 +838,17 @@
       <c r="A12" s="6" t="inlineStr"/>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>BUAD 310</t>
+          <t>ECON 352</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Applied Business Statistics</t>
+          <t>Macroeconomics for Business</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Marshall Core</t>
+          <t>Economics Requirement</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -823,6 +858,11 @@
       </c>
       <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Prereq ECON 351 (Fall 26)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr"/>
@@ -848,6 +888,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -857,12 +898,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>BUAD 311</t>
+          <t>BUAD 310</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Operations Management</t>
+          <t>Applied Business Statistics</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -883,6 +924,11 @@
       <c r="G14" s="6" t="inlineStr">
         <is>
           <t>102.0</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Stats moved here — not stacked with 306</t>
         </is>
       </c>
     </row>
@@ -890,17 +936,17 @@
       <c r="A15" s="4" t="inlineStr"/>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>WRIT 340</t>
+          <t>BUAD 311</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Advanced Writing</t>
+          <t>Operations Management</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Upper Division Writing</t>
+          <t>Marshall Core</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -910,22 +956,23 @@
       </c>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr"/>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>GE-E Course</t>
+          <t>WRIT 340</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Approved Physical Sciences Course</t>
+          <t>Advanced Writing</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>GE Category E</t>
+          <t>Upper Division Writing</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -935,6 +982,11 @@
       </c>
       <c r="F16" s="6" t="inlineStr"/>
       <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>STARS: still needed</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -972,6 +1024,7 @@
           <t>116.0</t>
         </is>
       </c>
+      <c r="H17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr"/>
@@ -997,6 +1050,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr"/>
       <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr"/>
@@ -1022,6 +1076,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr"/>
@@ -1047,6 +1102,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1084,6 +1140,7 @@
           <t>128.0</t>
         </is>
       </c>
+      <c r="H21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr"/>
@@ -1109,6 +1166,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr"/>
       <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr"/>
@@ -1134,10 +1192,11 @@
       </c>
       <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Swap REL 137 for HIST 103 and limit Spring 2027 to one Marshall course
Spring 2027: BUAD 302 + GE-C + ECON 352 (only BUAD 302 is Marshall).
Finance and stats moved to Fall 2027 and Spring 2028.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/graduation-plan.xlsx
+++ b/output/graduation-plan.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>In progress per STARS (08/15/26)</t>
+          <t>In progress per STARS</t>
         </is>
       </c>
     </row>
@@ -668,12 +668,12 @@
       <c r="A7" s="4" t="inlineStr"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>HIST 103</t>
+          <t>REL 137</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>The Emergence of Modern Europe</t>
+          <t>Intro to Islam</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -688,7 +688,11 @@
       </c>
       <c r="F7" s="4" t="inlineStr"/>
       <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Swapped from HIST 103 — still 4 units GE-B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -728,7 +732,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Rebalanced — lighter than finance/stats stack</t>
+          <t>Only 1 Marshall course this term (≤2 rule)</t>
         </is>
       </c>
     </row>
@@ -758,7 +762,7 @@
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Fulfills remaining GE-C; non-quant</t>
+          <t>Non-Marshall — fulfills remaining GE-C</t>
         </is>
       </c>
     </row>
@@ -766,17 +770,17 @@
       <c r="A10" s="6" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Elective</t>
+          <t>ECON 352</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>General Free Elective</t>
+          <t>Macroeconomics for Business</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Degree Units</t>
+          <t>Economics Requirement</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -788,7 +792,7 @@
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Buffer — keeps load at 12 not 15</t>
+          <t>Quant but NOT Marshall; prereq ECON 351</t>
         </is>
       </c>
     </row>
@@ -830,7 +834,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Quant course — paired with macro only</t>
+          <t>Single heavy Marshall term — finance only</t>
         </is>
       </c>
     </row>
@@ -838,17 +842,17 @@
       <c r="A12" s="6" t="inlineStr"/>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>ECON 352</t>
+          <t>GE-D Course</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Macroeconomics for Business</t>
+          <t>Approved Life Sciences Course</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Economics Requirement</t>
+          <t>GE Category D</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -858,27 +862,23 @@
       </c>
       <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Prereq ECON 351 (Fall 26)</t>
-        </is>
-      </c>
+      <c r="H12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>GE-D Course</t>
+          <t>Elective</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Approved Life Sciences Course</t>
+          <t>General Free Elective</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>GE Category D</t>
+          <t>Degree Units</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -888,7 +888,11 @@
       </c>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Light buffer alongside finance</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -928,7 +932,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Stats moved here — not stacked with 306</t>
+          <t>Stats + ops paired away from Spring 27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move BUAD 281 to Spring 2027 and add GE-D there
Fall 2026 drops to 12 units (304, ECON 351, REL 137). Spring 2027:
BUAD 281 + BUAD 302 + GE-C + GE-D (2 Marshall max). Fall 2027 loses
free elective; adds ECON 352 and WRIT 340 with BUAD 306.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/graduation-plan.xlsx
+++ b/output/graduation-plan.xlsx
@@ -578,37 +578,37 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>BUAD 281</t>
+          <t>BUAD 304</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Introduction to Managerial Accounting</t>
+          <t>Organizational Behavior and Leadership</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Accounting / Marshall Core</t>
+          <t>Marshall Core</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>In progress per STARS</t>
+          <t>BUAD 281 moved to Spring 2027</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>BUAD 304</t>
+          <t>ECON 351</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Organizational Behavior and Leadership</t>
+          <t>Microeconomics for Business</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Marshall Core</t>
+          <t>Economics / Marshall Core</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -642,17 +642,17 @@
       <c r="A6" s="6" t="inlineStr"/>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>ECON 351</t>
+          <t>REL 137</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Microeconomics for Business</t>
+          <t>Intro to Islam</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Economics / Marshall Core</t>
+          <t>GE Category B (Humanistic Inquiry)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -662,44 +662,56 @@
       </c>
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>4 units — swapped from HIST 103</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Spring 2027</t>
+        </is>
+      </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>REL 137</t>
+          <t>BUAD 281</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Intro to Islam</t>
+          <t>Introduction to Managerial Accounting</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>GE Category B (Humanistic Inquiry)</t>
+          <t>Accounting / Marshall Core</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Swapped from HIST 103 — still 4 units GE-B</t>
+          <t>Marshall #1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Spring 2027</t>
-        </is>
-      </c>
+      <c r="A8" s="6" t="inlineStr"/>
       <c r="B8" s="6" t="inlineStr">
         <is>
           <t>BUAD 302</t>
@@ -720,19 +732,11 @@
           <t>4.0</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>78.0</t>
-        </is>
-      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Only 1 Marshall course this term (≤2 rule)</t>
+          <t>Marshall #2 (≤2 rule met)</t>
         </is>
       </c>
     </row>
@@ -760,27 +764,23 @@
       </c>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Non-Marshall — fulfills remaining GE-C</t>
-        </is>
-      </c>
+      <c r="H9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>ECON 352</t>
+          <t>GE-D Course</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Macroeconomics for Business</t>
+          <t>Approved Life Sciences Course</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Economics Requirement</t>
+          <t>GE Category D</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -792,7 +792,7 @@
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Quant but NOT Marshall; prereq ECON 351</t>
+          <t>Replaces Fall 2027 free elective slot</t>
         </is>
       </c>
     </row>
@@ -832,27 +832,23 @@
           <t>90.0</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Single heavy Marshall term — finance only</t>
-        </is>
-      </c>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr"/>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>GE-D Course</t>
+          <t>ECON 352</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Approved Life Sciences Course</t>
+          <t>Macroeconomics for Business</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>GE Category D</t>
+          <t>Economics Requirement</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -862,23 +858,27 @@
       </c>
       <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Prereq ECON 351</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Elective</t>
+          <t>WRIT 340</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>General Free Elective</t>
+          <t>Advanced Writing</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Degree Units</t>
+          <t>Upper Division Writing</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -890,7 +890,7 @@
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Light buffer alongside finance</t>
+          <t>STARS: still needed</t>
         </is>
       </c>
     </row>
@@ -930,11 +930,7 @@
           <t>102.0</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>Stats + ops paired away from Spring 27</t>
-        </is>
-      </c>
+      <c r="H14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr"/>
@@ -966,17 +962,17 @@
       <c r="A16" s="6" t="inlineStr"/>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>WRIT 340</t>
+          <t>GE-E Course</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Advanced Writing</t>
+          <t>Approved Physical Sciences Course</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Upper Division Writing</t>
+          <t>GE Category E</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -986,11 +982,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr"/>
       <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>STARS: still needed</t>
-        </is>
-      </c>
+      <c r="H16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add GE-D consider column with Soultanakis HBIO-205/210 RMP research
Fetch and summarize Helen Soultanakis RMP reviews for HBIO-205 and HBIO-210,
and add a GE-D Consider column on the graduation plan pointing to these
exam-only Life Sciences options.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/graduation-plan.xlsx
+++ b/output/graduation-plan.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -497,6 +497,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -547,6 +548,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>GE-D Consider (Prof / Class)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -795,6 +801,11 @@
           <t>Replaces Fall 2027 free elective slot</t>
         </is>
       </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>HBIO-205 Science of Sport · Prof. Soultanakis (Fall sec 38411) · HBIO-210 Mediterranean Lifestyles · Prof. Soultanakis (Fall sec 38452) · RMP 2.8 quality / 2.8 difficulty · no papers · 2 MC midterms (drop lower) + MC final · memorize slides/study guides</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1192,7 +1203,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Move WRIT 340 from Fall 2027 to Fall 2028 in graduation plan
Shift Advanced Writing to senior fall and backfill Fall 2027 with a free
elective so the term stays at 12 units.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/graduation-plan.xlsx
+++ b/output/graduation-plan.xlsx
@@ -843,7 +843,11 @@
           <t>90.0</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>WRIT 340 moved to Fall 2028</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr"/>
@@ -879,17 +883,17 @@
       <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>WRIT 340</t>
+          <t>Elective</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Advanced Writing</t>
+          <t>General Free Elective</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Upper Division Writing</t>
+          <t>Degree Units</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -901,7 +905,7 @@
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>STARS: still needed</t>
+          <t>Moved from Fall 2028 to keep 12 units</t>
         </is>
       </c>
     </row>
@@ -1089,17 +1093,17 @@
       <c r="A20" s="6" t="inlineStr"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Elective</t>
+          <t>WRIT 340</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>General Free Elective</t>
+          <t>Advanced Writing</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Degree Units</t>
+          <t>Upper Division Writing</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1109,7 +1113,11 @@
       </c>
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Moved from Fall 2027 — STARS: still needed</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add Professor Notes to ANTH-202 workbook tab with Mayfield RMP essay data
- build_workbook: render professor_notes dict on class sheets
- anth202.json: syllabus + RMP midterm prep and essay grading quotes
- rmp.json: essay_grading_reviews array with 17 curated ANTH-202 quotes
- Rebuild syllabi.xlsx and graduation-plan.xlsx

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/graduation-plan.xlsx
+++ b/output/graduation-plan.xlsx
@@ -750,12 +750,12 @@
       <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>GE-C Course</t>
+          <t>ANTH 202</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Approved Social Analysis (e.g. ANTH 202)</t>
+          <t>Archaeology: Our Human Past</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -770,7 +770,11 @@
       </c>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Prof. Tracie Mayfield · RMP 4.6 quality / 2.1 difficulty · 82% would take again · avg grade A- (3.93 GPA) · open-book midterm/final (MC mostly from weekly quizzes) · final paper built via worksheets + peer review · reviews: prepares well for exams, generally lenient grader if you keep up</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr"/>
@@ -971,7 +975,11 @@
       </c>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Preferred: Charlie Hannigan (14911 8am MW or 14913 9:30am MW) · RMP 4.7 / diff 2.7 · 2024 Golden Apple · easiest A odds on roster; avoid Takayama if possible (only open sections)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr"/>

</xml_diff>